<commit_message>
implemented redirect check and spell check
</commit_message>
<xml_diff>
--- a/tests/PageVerificationUrls.xlsx
+++ b/tests/PageVerificationUrls.xlsx
@@ -38,7 +38,7 @@
     <t>https://www.softwebsolutions.com/python-development-services/</t>
   </si>
   <si>
-    <t>https://www.softwebsolutions.com/quality-inspection-in-manufacturing/</t>
+    <t>https://www.softwebsolutions.com/quality-inspect</t>
   </si>
 </sst>
 </file>
@@ -1071,10 +1071,13 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="https://www.softwebsolutions.com/quality-inspect" tooltip="https://www.softwebsolutions.com/quality-inspect"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A2:A4" numberStoredAsText="1"/>
+    <ignoredError sqref="A2:A3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added dependency of spell check in launh bat
</commit_message>
<xml_diff>
--- a/tests/PageVerificationUrls.xlsx
+++ b/tests/PageVerificationUrls.xlsx
@@ -38,7 +38,7 @@
     <t>https://www.softwebsolutions.com/python-development-services/</t>
   </si>
   <si>
-    <t>https://www.softwebsolutions.com/quality-inspect</t>
+    <t>https://www.softwebsolutions.com/quality-inspect/</t>
   </si>
 </sst>
 </file>
@@ -1072,7 +1072,7 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A4" r:id="rId1" display="https://www.softwebsolutions.com/quality-inspect" tooltip="https://www.softwebsolutions.com/quality-inspect"/>
+    <hyperlink ref="A4" r:id="rId1" display="https://www.softwebsolutions.com/quality-inspect/" tooltip="https://www.softwebsolutions.com/quality-inspect/"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>